<commit_message>
Add site oficial do mestrado ao faq e docs
</commit_message>
<xml_diff>
--- a/base_perguntas_respostas_ppgd.xlsx
+++ b/base_perguntas_respostas_ppgd.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perguntas_Respostas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fallback" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Perguntas_Respostas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fallback" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fontes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumo" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Perguntas_Respostas'!$A$1:$J$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Perguntas_Respostas'!$A$1:$J$245</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fallback'!$A$1:$E$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fontes'!$A$1:$C$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Resumo'!$A$1:$B$6</definedName>
@@ -148,8 +148,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaPerguntasRespostas" displayName="TabelaPerguntasRespostas" ref="A1:J170" headerRowCount="1">
-  <autoFilter ref="A1:J170"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaPerguntasRespostas" displayName="TabelaPerguntasRespostas" ref="A1:J245" headerRowCount="1">
+  <autoFilter ref="A1:J245"/>
   <tableColumns count="10">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="categoria"/>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J170"/>
+  <dimension ref="A1:J245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9157,47 +9157,47 @@
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>fallback_mensalidade_01</t>
+          <t>q046_01</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>curriculo_disciplinas</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>fora_da_base</t>
+          <t>qual_a_ementa_da_disciplina_de_processo_penal_e_</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Qual é o valor da mensalidade?</t>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Quanto custa o mestrado?</t>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+          <t>A ementa engloba os seguintes tópicos: O processo penal no contexto criminal e seus discursos (pós-CF/88), Princípios, garantias constitucionais e a aplicação pelos Tribunais Superiores, Investigação preliminar e a investigação defensiva, Crítica à Teoria Geral do Processo (jurisdição, ação e processo), A verdade, a prova lícita e ilícita, Medidas cautelares e o poder geral de cautela, Reformas na América Latina e o novo Código de Processo Penal, Justiça negocial e sua expansão, Práticas no sistema criminal “pós operação Lava-Jato”.</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>Sem informação nos documentos analisados</t>
+          <t>`docs/texts/ementas_disciplinas.txt`.</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>rag</t>
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>Onde acompanho publicações do mestrado?</t>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -9209,47 +9209,47 @@
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>fallback_edital_01</t>
+          <t>q046_02</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>curriculo_disciplinas</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>edital_atual</t>
+          <t>qual_a_ementa_da_disciplina_de_processo_penal_e_</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>Quando abre inscrição para a próxima turma?</t>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>Qual a data do próximo edital?</t>
+          <t>Gostaria de saber: qual a ementa da disciplina de processo penal e prática judiciária?</t>
         </is>
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta com segurança. Para editais e notícias, consulte as publicações oficiais do Mestrado.</t>
+          <t>A ementa engloba os seguintes tópicos: O processo penal no contexto criminal e seus discursos (pós-CF/88), Princípios, garantias constitucionais e a aplicação pelos Tribunais Superiores, Investigação preliminar e a investigação defensiva, Crítica à Teoria Geral do Processo (jurisdição, ação e processo), A verdade, a prova lícita e ilícita, Medidas cautelares e o poder geral de cautela, Reformas na América Latina e o novo Código de Processo Penal, Justiça negocial e sua expansão, Práticas no sistema criminal “pós operação Lava-Jato”.</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>Sem calendário atual nos documentos analisados</t>
+          <t>`docs/texts/ementas_disciplinas.txt`.</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
-          <t>fallback</t>
+          <t>rag</t>
         </is>
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>Onde acompanho publicações do mestrado?</t>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr">
@@ -9261,57 +9261,3957 @@
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
+          <t>q046_03</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_ementa_da_disciplina_de_processo_penal_e_</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual a ementa da disciplina de processo penal e prática judiciária?</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>A ementa engloba os seguintes tópicos: O processo penal no contexto criminal e seus discursos (pós-CF/88), Princípios, garantias constitucionais e a aplicação pelos Tribunais Superiores, Investigação preliminar e a investigação defensiva, Crítica à Teoria Geral do Processo (jurisdição, ação e processo), A verdade, a prova lícita e ilícita, Medidas cautelares e o poder geral de cautela, Reformas na América Latina e o novo Código de Processo Penal, Justiça negocial e sua expansão, Práticas no sistema criminal “pós operação Lava-Jato”.</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/ementas_disciplinas.txt`.</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa da disciplina de Processo Penal e Prática Judiciária?</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>q047_01</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_ementa_completa_da_disciplina_de_promoção</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>A ementa aborda: Poder Judiciário no Estado e Judicialização da Política/Políticas Sociais, Juristocracia, Politização e Judicialização dos Direitos Coletivos, Limites e legitimidade da atuação do Poder Judiciário, Controle da Administração Pública e Constitucionalidade das Políticas Públicas, A jurisprudência do STF: decisões entre teorias constitucionais e governabilidade.</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/ementas_disciplinas.txt`.</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>q047_02</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_ementa_completa_da_disciplina_de_promoção</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: qual a ementa completa da disciplina de promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>A ementa aborda: Poder Judiciário no Estado e Judicialização da Política/Políticas Sociais, Juristocracia, Politização e Judicialização dos Direitos Coletivos, Limites e legitimidade da atuação do Poder Judiciário, Controle da Administração Pública e Constitucionalidade das Políticas Públicas, A jurisprudência do STF: decisões entre teorias constitucionais e governabilidade.</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/ementas_disciplinas.txt`.</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>q047_03</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_ementa_completa_da_disciplina_de_promoção</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual a ementa completa da disciplina de promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>A ementa aborda: Poder Judiciário no Estado e Judicialização da Política/Políticas Sociais, Juristocracia, Politização e Judicialização dos Direitos Coletivos, Limites e legitimidade da atuação do Poder Judiciário, Controle da Administração Pública e Constitucionalidade das Políticas Públicas, A jurisprudência do STF: decisões entre teorias constitucionais e governabilidade.</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/ementas_disciplinas.txt`.</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>Qual a ementa completa da disciplina de Promoção de políticas públicas e judicialização?</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>q048_01</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>será_que_consigo_aproveitamento_numa_disciplina_</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>Sim. Admite-se o aproveitamento de disciplinas cursadas nos formatos presencial, remoto ou híbrido.</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n.-8-2024-sobre-aproveitamento-de-disciplinas-01-10-2024.pdf`.</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>q048_02</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>será_que_consigo_aproveitamento_numa_disciplina_</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>Sim. Admite-se o aproveitamento de disciplinas cursadas nos formatos presencial, remoto ou híbrido.</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n.-8-2024-sobre-aproveitamento-de-disciplinas-01-10-2024.pdf`.</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>q048_03</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>será_que_consigo_aproveitamento_numa_disciplina_</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Sim. Admite-se o aproveitamento de disciplinas cursadas nos formatos presencial, remoto ou híbrido.</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n.-8-2024-sobre-aproveitamento-de-disciplinas-01-10-2024.pdf`.</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>Será que consigo aproveitamento numa disciplina que fiz no modelo remoto?</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>q049_01</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_pontuação_mínima_no_exame_michigan_ecce_p</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>A pontuação mínima exigida neste exame é de 650 pontos.</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>q049_02</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_pontuação_mínima_no_exame_michigan_ecce_p</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: qual a pontuação mínima no exame michigan ecce para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>A pontuação mínima exigida neste exame é de 650 pontos.</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>q049_03</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_pontuação_mínima_no_exame_michigan_ecce_p</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual a pontuação mínima no exame michigan ecce para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>A pontuação mínima exigida neste exame é de 650 pontos.</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no exame Michigan ECCE para comprovação de língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>q050_01</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_teap_é_aceito_pela_pós_como_suficiência_</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Sim. A pontuação mínima exigida no TEAP é de 70 pontos.</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>q050_02</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_teap_é_aceito_pela_pós_como_suficiência_</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>Sim. A pontuação mínima exigida no TEAP é de 70 pontos.</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>q050_03</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_teap_é_aceito_pela_pós_como_suficiência_</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: o exame teap é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>Sim. A pontuação mínima exigida no TEAP é de 70 pontos.</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>q050_04</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_teap_é_aceito_pela_pós_como_suficiência_</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder o exame teap é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr">
+        <is>
+          <t>Sim. A pontuação mínima exigida no TEAP é de 70 pontos.</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>O exame TEAP é aceito pela pós como suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>q051_01</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>defesa_documentos</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>o_que_deve_conter_a_introdução_ampliada_na_disse</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr">
+        <is>
+          <t>A introdução ampliada deve ter entre 3 e 10 páginas (podendo conter subtópicos) e incluir obrigatoriamente: O estado da arte, as justificativas da pesquisa, as hipóteses da pesquisa.</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>q051_02</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>defesa_documentos</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>o_que_deve_conter_a_introdução_ampliada_na_disse</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr">
+        <is>
+          <t>A introdução ampliada deve ter entre 3 e 10 páginas (podendo conter subtópicos) e incluir obrigatoriamente: O estado da arte, as justificativas da pesquisa, as hipóteses da pesquisa.</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>q051_03</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>defesa_documentos</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>o_que_deve_conter_a_introdução_ampliada_na_disse</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: o que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>A introdução ampliada deve ter entre 3 e 10 páginas (podendo conter subtópicos) e incluir obrigatoriamente: O estado da arte, as justificativas da pesquisa, as hipóteses da pesquisa.</t>
+        </is>
+      </c>
+      <c r="G186" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>q051_04</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>defesa_documentos</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>o_que_deve_conter_a_introdução_ampliada_na_disse</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder o que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>A introdução ampliada deve ter entre 3 e 10 páginas (podendo conter subtópicos) e incluir obrigatoriamente: O estado da arte, as justificativas da pesquisa, as hipóteses da pesquisa.</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>O que deve conter a introdução ampliada na dissertação de formato escandinavo?</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>q052_01</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>na_qualificação_da_dissertação_escandinava_preci</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>Não nesta etapa. O documento de qualificação no modelo alternativo deve apresentar apenas: Elementos básicos: Capa, contracapa, banca, resumo, abstract e sumário, Corpo principal: Introdução, metodologia e eventuais artigos (concluídos ou em andamento), Produto: Descrição do produto translacional.</t>
+        </is>
+      </c>
+      <c r="G188" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>q052_02</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>na_qualificação_da_dissertação_escandinava_preci</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>Não nesta etapa. O documento de qualificação no modelo alternativo deve apresentar apenas: Elementos básicos: Capa, contracapa, banca, resumo, abstract e sumário, Corpo principal: Introdução, metodologia e eventuais artigos (concluídos ou em andamento), Produto: Descrição do produto translacional.</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>q052_03</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>na_qualificação_da_dissertação_escandinava_preci</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Não nesta etapa. O documento de qualificação no modelo alternativo deve apresentar apenas: Elementos básicos: Capa, contracapa, banca, resumo, abstract e sumário, Corpo principal: Introdução, metodologia e eventuais artigos (concluídos ou em andamento), Produto: Descrição do produto translacional.</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>`INSTRUCAO-NORMATIVA-09.2025.pdf`.</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>Na qualificação da dissertação escandinava, preciso já incluir as considerações finais?</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>q053_01</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>até_quando_as_vagas_de_fomento_podem_ser_ofertad</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>As vagas são definidas até o mês de agosto de cada ano letivo, quando o Coordenador relata ao Colegiado o interesse das instituições parceiras e avalia os requisitos.</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>`IN-Normativa-12-2025-Vagas-de-Fomento-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>q053_02</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>até_quando_as_vagas_de_fomento_podem_ser_ofertad</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>As vagas são definidas até o mês de agosto de cada ano letivo, quando o Coordenador relata ao Colegiado o interesse das instituições parceiras e avalia os requisitos.</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>`IN-Normativa-12-2025-Vagas-de-Fomento-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>q053_03</t>
+        </is>
+      </c>
+      <c r="B193" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>até_quando_as_vagas_de_fomento_podem_ser_ofertad</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="E193" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr">
+        <is>
+          <t>As vagas são definidas até o mês de agosto de cada ano letivo, quando o Coordenador relata ao Colegiado o interesse das instituições parceiras e avalia os requisitos.</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>`IN-Normativa-12-2025-Vagas-de-Fomento-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>Até quando as vagas de fomento podem ser ofertadas?</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>q054_01</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>como_fica_o_prazo_do_mestrado_em_caso_de_comprom</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr">
+        <is>
+          <t>Os impactos nos prazos por motivo de saúde são analisados caso a caso pelo Colegiado do Programa. O que fazer: Comunique formalmente a sua condição ao seu Orientador(a) e ao Colegiado o mais breve possível.</t>
+        </is>
+      </c>
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>q054_02</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>como_fica_o_prazo_do_mestrado_em_caso_de_comprom</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="E195" s="2" t="inlineStr">
+        <is>
+          <t>De que forma fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>Os impactos nos prazos por motivo de saúde são analisados caso a caso pelo Colegiado do Programa. O que fazer: Comunique formalmente a sua condição ao seu Orientador(a) e ao Colegiado o mais breve possível.</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>q054_03</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>como_fica_o_prazo_do_mestrado_em_caso_de_comprom</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr">
+        <is>
+          <t>Os impactos nos prazos por motivo de saúde são analisados caso a caso pelo Colegiado do Programa. O que fazer: Comunique formalmente a sua condição ao seu Orientador(a) e ao Colegiado o mais breve possível.</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>q054_04</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>como_fica_o_prazo_do_mestrado_em_caso_de_comprom</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t>Os impactos nos prazos por motivo de saúde são analisados caso a caso pelo Colegiado do Programa. O que fazer: Comunique formalmente a sua condição ao seu Orientador(a) e ao Colegiado o mais breve possível.</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>Como fica o prazo do mestrado em caso de comprometimento de saúde (ex: acidentes)?</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>q055_01</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>existe_período_mínimo_de_atestado_para_solicitar</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>Sim. O RED não se aplica para atestados ou licenças inferiores a 15 dias.</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>q055_02</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>existe_período_mínimo_de_atestado_para_solicitar</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: existe período mínimo de atestado para solicitar o regime de exercícios domiciliares (red)?</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>Sim. O RED não se aplica para atestados ou licenças inferiores a 15 dias.</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>q055_03</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>existe_período_mínimo_de_atestado_para_solicitar</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder existe período mínimo de atestado para solicitar o regime de exercícios domiciliares (red)?</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Sim. O RED não se aplica para atestados ou licenças inferiores a 15 dias.</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>Existe período mínimo de atestado para solicitar o Regime de Exercícios Domiciliares (RED)?</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>q056_01</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>sou_mestranda_bolsista_da_capes_em_caso_de_gravi</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Não. Os pagamentos não são suspensos durante a licença-maternidade. Porém, é necessário: Comunicar formalmente o afastamento à CAPES, enviar a confirmação da PROPESP (com datas exatas de início e fim), apresentar os documentos comprobatórios (gestação e nascimento).</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>q056_02</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>sou_mestranda_bolsista_da_capes_em_caso_de_gravi</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: sou mestranda bolsista da capes, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>Não. Os pagamentos não são suspensos durante a licença-maternidade. Porém, é necessário: Comunicar formalmente o afastamento à CAPES, enviar a confirmação da PROPESP (com datas exatas de início e fim), apresentar os documentos comprobatórios (gestação e nascimento).</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>q056_03</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>sou_mestranda_bolsista_da_capes_em_caso_de_gravi</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder sou mestranda bolsista da capes, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>Não. Os pagamentos não são suspensos durante a licença-maternidade. Porém, é necessário: Comunicar formalmente o afastamento à CAPES, enviar a confirmação da PROPESP (com datas exatas de início e fim), apresentar os documentos comprobatórios (gestação e nascimento).</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>Sou mestranda bolsista da CAPES, em caso de gravidez eu perco a bolsa?</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>q057_01</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>quantos_créditos_valem_o_estágio_de_docência</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>O estágio de docência vale ao todo 2 créditos.</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>`TABELA-ATIVIDADES-COMPLEMNTARES-IN-05.2024-ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>q057_02</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>quantos_créditos_valem_o_estágio_de_docência</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>O estágio de docência vale ao todo 2 créditos.</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>`TABELA-ATIVIDADES-COMPLEMNTARES-IN-05.2024-ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>q057_03</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>curriculo_disciplinas</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>quantos_créditos_valem_o_estágio_de_docência</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>O estágio de docência vale ao todo 2 créditos.</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t>`TABELA-ATIVIDADES-COMPLEMNTARES-IN-05.2024-ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>Quantos créditos valem o estágio de docência?</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>q058_01</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>são_quantas_horas_totais_de_estágio_de_imersão_p</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>O estágio exige um total de 60 horas.</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>q058_02</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>são_quantas_horas_totais_de_estágio_de_imersão_p</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: são quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>O estágio exige um total de 60 horas.</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>q058_03</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>são_quantas_horas_totais_de_estágio_de_imersão_p</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder são quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>O estágio exige um total de 60 horas.</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t>São quantas horas totais de estágio de imersão prático-institucional?</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>q059_01</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>é_permitido_realizar_o_estágio_prático_instituci</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>Sim, desde que seja compatível com a sua pesquisa e carga horária. É obrigatório: Apresentar Termos de Compromisso e Declarações de Horas separados para cada local, citar a pluralidade de locais no seu projeto, no relatório final e no seminário.</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>q059_02</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>é_permitido_realizar_o_estágio_prático_instituci</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: é permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>Sim, desde que seja compatível com a sua pesquisa e carga horária. É obrigatório: Apresentar Termos de Compromisso e Declarações de Horas separados para cada local, citar a pluralidade de locais no seu projeto, no relatório final e no seminário.</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>q059_03</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>é_permitido_realizar_o_estágio_prático_instituci</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder é permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>Sim, desde que seja compatível com a sua pesquisa e carga horária. É obrigatório: Apresentar Termos de Compromisso e Declarações de Horas separados para cada local, citar a pluralidade de locais no seu projeto, no relatório final e no seminário.</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n-5-2024-Atividades-complementares-24-06-2024-atualizada-pela-IN-07-2024ATUALIZADA.pdf`.</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>É permitido realizar o estágio prático-institucional em mais de um lugar no mesmo período?</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>q060_01</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>como_faço_para_agendar_o_uso_e_pegar_a_chave_do_</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>O agendamento é feito na Secretaria do PPGD (Segunda a sexta, das 08h30 às 17h30). Prazo: Mínimo de 7 dias de antecedência, Exceção: O prazo pode ser menor caso você não vá utilizar os equipamentos tecnológicos/audiovisuais do laboratório.</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>`Proposta-Ordem-de-Seviço-Laboratório-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>q060_02</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>como_faço_para_agendar_o_uso_e_pegar_a_chave_do_</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>De que forma faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>O agendamento é feito na Secretaria do PPGD (Segunda a sexta, das 08h30 às 17h30). Prazo: Mínimo de 7 dias de antecedência, Exceção: O prazo pode ser menor caso você não vá utilizar os equipamentos tecnológicos/audiovisuais do laboratório.</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t>`Proposta-Ordem-de-Seviço-Laboratório-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>q060_03</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>como_faço_para_agendar_o_uso_e_pegar_a_chave_do_</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>O agendamento é feito na Secretaria do PPGD (Segunda a sexta, das 08h30 às 17h30). Prazo: Mínimo de 7 dias de antecedência, Exceção: O prazo pode ser menor caso você não vá utilizar os equipamentos tecnológicos/audiovisuais do laboratório.</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t>`Proposta-Ordem-de-Seviço-Laboratório-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>q060_04</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>como_faço_para_agendar_o_uso_e_pegar_a_chave_do_</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>O agendamento é feito na Secretaria do PPGD (Segunda a sexta, das 08h30 às 17h30). Prazo: Mínimo de 7 dias de antecedência, Exceção: O prazo pode ser menor caso você não vá utilizar os equipamentos tecnológicos/audiovisuais do laboratório.</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t>`Proposta-Ordem-de-Seviço-Laboratório-1.pdf`.</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>Como faço para agendar o uso e pegar a chave do laboratório da pós?</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>q061_01</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_site_do_setor_de_ciências_jurídicas_sec</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é: https://www2.uepg.br/direito/setor-de-ciencias-juridicas/</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/contatos.txt`.</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>q061_02</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_site_do_setor_de_ciências_jurídicas_sec</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t>Me informe o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é: https://www2.uepg.br/direito/setor-de-ciencias-juridicas/</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/contatos.txt`.</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>q061_03</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_site_do_setor_de_ciências_jurídicas_sec</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: qual é o site do setor de ciências jurídicas (secijur)?</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é: https://www2.uepg.br/direito/setor-de-ciencias-juridicas/</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/contatos.txt`.</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>q061_04</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_site_do_setor_de_ciências_jurídicas_sec</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual é o site do setor de ciências jurídicas (secijur)?</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é: https://www2.uepg.br/direito/setor-de-ciencias-juridicas/</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t>`docs/texts/contatos.txt`.</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o site do Setor de Ciências Jurídicas (SECIJUR)?</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>q062_01</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_pontuação_mínima_no_ielts_para_comprovar_</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t>A pontuação mínima a ser atingida no exame é 6 pontos.</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>q062_02</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_pontuação_mínima_no_ielts_para_comprovar_</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: qual a pontuação mínima no ielts para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>A pontuação mínima a ser atingida no exame é 6 pontos.</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>q062_03</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>qual_a_pontuação_mínima_no_ielts_para_comprovar_</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual a pontuação mínima no ielts para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>A pontuação mínima a ser atingida no exame é 6 pontos.</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>Qual a pontuação mínima no IELTS para comprovar suficiência em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>q063_01</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_cambridge_esol_skills_for_life_pode_ser_</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>Sim, portanto que o resultado atingido seja "Pass".</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>q063_02</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_cambridge_esol_skills_for_life_pode_ser_</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t>exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>Sim, portanto que o resultado atingido seja "Pass".</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>q063_03</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_cambridge_esol_skills_for_life_pode_ser_</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: o exame cambridge esol skills for life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>Sim, portanto que o resultado atingido seja "Pass".</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>q063_04</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>o_exame_cambridge_esol_skills_for_life_pode_ser_</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder o exame cambridge esol skills for life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>Sim, portanto que o resultado atingido seja "Pass".</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>`Instrucao-Normativa-n°-10-suficiencia-em-linguas.pdf`.</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>O exame Cambridge ESOL Skills for Life pode ser aceito para comprovação em língua estrangeira?</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>q064_01</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_prazo_para_entregar_o_atestado_e_solici</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>O prazo máximo para protocolar o atestado médico ou odontológico no Protocolo Geral da UEPG é de 3 dias úteis. A contagem desse prazo se inicia na data de emissão que consta no atestado. Pedidos realizados com atraso ou com falta de documentos serão indeferidos.</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>q064_02</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_prazo_para_entregar_o_atestado_e_solici</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="inlineStr">
+        <is>
+          <t>Me informe o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>O prazo máximo para protocolar o atestado médico ou odontológico no Protocolo Geral da UEPG é de 3 dias úteis. A contagem desse prazo se inicia na data de emissão que consta no atestado. Pedidos realizados com atraso ou com falta de documentos serão indeferidos.</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>q064_03</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_prazo_para_entregar_o_atestado_e_solici</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: qual é o prazo para entregar o atestado e solicitar o red?</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>O prazo máximo para protocolar o atestado médico ou odontológico no Protocolo Geral da UEPG é de 3 dias úteis. A contagem desse prazo se inicia na data de emissão que consta no atestado. Pedidos realizados com atraso ou com falta de documentos serão indeferidos.</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>q064_04</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr">
+        <is>
+          <t>prazos_requisitos</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>qual_é_o_prazo_para_entregar_o_atestado_e_solici</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual é o prazo para entregar o atestado e solicitar o red?</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>O prazo máximo para protocolar o atestado médico ou odontológico no Protocolo Geral da UEPG é de 3 dias úteis. A contagem desse prazo se inicia na data de emissão que consta no atestado. Pedidos realizados com atraso ou com falta de documentos serão indeferidos.</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o prazo para entregar o atestado e solicitar o RED?</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>q065_01</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>o_red_pode_ser_usado_para_justificar_faltas_em_q</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>Não. O Regime de Exercícios Domiciliares não se aplica nas seguintes situações: Estágios curriculares obrigatórios, práticas laboratoriais e componentes que exijam a presença física do discente. Sessões de Exame de Qualificação, Seminários e bancas de Defesa de Dissertação. Quando o discente já tiver extrapolado o limite máximo de faltas permitido na disciplina.</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>q065_02</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>o_red_pode_ser_usado_para_justificar_faltas_em_q</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="inlineStr">
+        <is>
+          <t>RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>Não. O Regime de Exercícios Domiciliares não se aplica nas seguintes situações: Estágios curriculares obrigatórios, práticas laboratoriais e componentes que exijam a presença física do discente. Sessões de Exame de Qualificação, Seminários e bancas de Defesa de Dissertação. Quando o discente já tiver extrapolado o limite máximo de faltas permitido na disciplina.</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I233" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>q065_03</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>o_red_pode_ser_usado_para_justificar_faltas_em_q</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: o red pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>Não. O Regime de Exercícios Domiciliares não se aplica nas seguintes situações: Estágios curriculares obrigatórios, práticas laboratoriais e componentes que exijam a presença física do discente. Sessões de Exame de Qualificação, Seminários e bancas de Defesa de Dissertação. Quando o discente já tiver extrapolado o limite máximo de faltas permitido na disciplina.</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>q065_04</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr">
+        <is>
+          <t>normas_procedimentos</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>o_red_pode_ser_usado_para_justificar_faltas_em_q</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder o red pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>Não. O Regime de Exercícios Domiciliares não se aplica nas seguintes situações: Estágios curriculares obrigatórios, práticas laboratoriais e componentes que exijam a presença física do discente. Sessões de Exame de Qualificação, Seminários e bancas de Defesa de Dissertação. Quando o discente já tiver extrapolado o limite máximo de faltas permitido na disciplina.</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>`2018-08-21_Resolucao-CEPE-043-RED.pdf`.</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>O RED pode ser usado para justificar faltas em qualquer atividade do mestrado?</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>q066_01</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>o_que_é_a_uepg</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>A Universidade Estadual de Ponta Grossa é uma das mais respeitadas instituições de ensino público e gratuito do Brasil, sendo a instituição de ensino superior de maior impacto regional. Está localizada no sul do país, em Ponta Grossa, cidade que é importante polo de desenvolvimento dos Campos Gerais, região com 19 municípios. Com mais de 50 anos, a UEPG é um complexo que forma estudantes na educação básica, ensino médio, graduação e pós-graduação.</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>`https://www.uepg.br/sobre-a-uepg/`.</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>q066_02</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>o_que_é_a_uepg</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="inlineStr">
+        <is>
+          <t>Explique a UEPG?</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>A Universidade Estadual de Ponta Grossa é uma das mais respeitadas instituições de ensino público e gratuito do Brasil, sendo a instituição de ensino superior de maior impacto regional. Está localizada no sul do país, em Ponta Grossa, cidade que é importante polo de desenvolvimento dos Campos Gerais, região com 19 municípios. Com mais de 50 anos, a UEPG é um complexo que forma estudantes na educação básica, ensino médio, graduação e pós-graduação.</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>`https://www.uepg.br/sobre-a-uepg/`.</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>q066_03</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>o_que_é_a_uepg</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: o que é a uepg?</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>A Universidade Estadual de Ponta Grossa é uma das mais respeitadas instituições de ensino público e gratuito do Brasil, sendo a instituição de ensino superior de maior impacto regional. Está localizada no sul do país, em Ponta Grossa, cidade que é importante polo de desenvolvimento dos Campos Gerais, região com 19 municípios. Com mais de 50 anos, a UEPG é um complexo que forma estudantes na educação básica, ensino médio, graduação e pós-graduação.</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>`https://www.uepg.br/sobre-a-uepg/`.</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>q066_04</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>o_que_é_a_uepg</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder o que é a uepg?</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>A Universidade Estadual de Ponta Grossa é uma das mais respeitadas instituições de ensino público e gratuito do Brasil, sendo a instituição de ensino superior de maior impacto regional. Está localizada no sul do país, em Ponta Grossa, cidade que é importante polo de desenvolvimento dos Campos Gerais, região com 19 municípios. Com mais de 50 anos, a UEPG é um complexo que forma estudantes na educação básica, ensino médio, graduação e pós-graduação.</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>`https://www.uepg.br/sobre-a-uepg/`.</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>O que é a UEPG?</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>q067_01</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>qual_o_site_oficial_do_mestrado</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é https://www2.uepg.br/direito/mestrado/</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>`https://www2.uepg.br/direito/mestrado/`</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>q067_02</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>qual_o_site_oficial_do_mestrado</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="inlineStr">
+        <is>
+          <t>Gostaria de saber: qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é https://www2.uepg.br/direito/mestrado/</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>`https://www2.uepg.br/direito/mestrado/`</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>q067_03</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>programa</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>qual_o_site_oficial_do_mestrado</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>Você pode me responder qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>O site oficial é https://www2.uepg.br/direito/mestrado/</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>`https://www2.uepg.br/direito/mestrado/`</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>rag</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>Qual o site oficial do mestrado?</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>fallback_mensalidade_01</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>fora_da_base</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>Qual é o valor da mensalidade?</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>Quanto custa o mestrado?</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>Sem informação nos documentos analisados</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>Onde acompanho publicações do mestrado?</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>fallback_edital_01</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>edital_atual</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>Quando abre inscrição para a próxima turma?</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>Qual a data do próximo edital?</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta com segurança. Para editais e notícias, consulte as publicações oficiais do Mestrado.</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>Sem calendário atual nos documentos analisados</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>Onde acompanho publicações do mestrado?</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
           <t>fallback_ambigua_01</t>
         </is>
       </c>
-      <c r="B170" s="2" t="inlineStr">
+      <c r="B245" s="2" t="inlineStr">
         <is>
           <t>fallback</t>
         </is>
       </c>
-      <c r="C170" s="2" t="inlineStr">
+      <c r="C245" s="2" t="inlineStr">
         <is>
           <t>pergunta_ambigua</t>
         </is>
       </c>
-      <c r="D170" s="2" t="inlineStr">
+      <c r="D245" s="2" t="inlineStr">
         <is>
           <t>Qual é o prazo?</t>
         </is>
       </c>
-      <c r="E170" s="2" t="inlineStr">
+      <c r="E245" s="2" t="inlineStr">
         <is>
           <t>E isso, como funciona?</t>
         </is>
       </c>
-      <c r="F170" s="2" t="inlineStr">
+      <c r="F245" s="2" t="inlineStr">
         <is>
           <t>Você poderia reformular a pergunta informando o tema? Posso ajudar com prazos de conclusão, qualificação, defesa, disciplinas, créditos, suficiência ou atividades complementares.</t>
         </is>
       </c>
-      <c r="G170" s="2" t="inlineStr">
+      <c r="G245" s="2" t="inlineStr">
         <is>
           <t>Resposta padrão para baixa confiança</t>
         </is>
       </c>
-      <c r="H170" s="2" t="inlineStr">
+      <c r="H245" s="2" t="inlineStr">
         <is>
           <t>fallback</t>
         </is>
       </c>
-      <c r="I170" s="2" t="inlineStr">
+      <c r="I245" s="2" t="inlineStr">
         <is>
           <t>Qual o prazo para entregar a versão final após a defesa?</t>
         </is>
       </c>
-      <c r="J170" s="2" t="inlineStr">
+      <c r="J245" s="2" t="inlineStr">
         <is>
           <t>Desculpe, não tenho informações suficientes para responder a essa pergunta. Posso tentar ajudar com informações sobre prazos, disciplinas, créditos, defesa, suficiência, atividades complementares, documentos, contatos ou links do Programa.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J170"/>
+  <autoFilter ref="A1:J245"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10174,7 +14074,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>169</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3">
@@ -10184,7 +14084,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4">

</xml_diff>